<commit_message>
fix: correct narrow-gauge visitor verification status and revise README rationale
修订README"研究范围说明"
</commit_message>
<xml_diff>
--- a/data/raw/taian_indicators.xlsx
+++ b/data/raw/taian_indicators.xlsx
@@ -41,7 +41,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,11 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -79,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -95,6 +100,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1473,13 +1481,13 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <v>567.9</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="9" t="n">
         <v>278.6</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="9" t="n">
         <v>331.7</v>
       </c>
       <c r="I8" s="4" t="n">
@@ -1488,7 +1496,7 @@
       <c r="J8" s="4" t="n">
         <v>861.97</v>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="K8" s="9" t="n">
         <v>806.29</v>
       </c>
       <c r="L8" s="8" t="n">
@@ -1496,7 +1504,8 @@
       </c>
       <c r="M8" s="8" t="inlineStr">
         <is>
-          <t>【口径:进山/进泰山,不含非登顶访客】2019、2021年公报用词"进山进景点游客",2024、2025年用词"进泰山/进山游客量";2020年原文用词已核实(2026-08-26,PDF公报原文确认为"进山进景点游客278.6万",与主序列一致);2022、2023年公报未披露,仍为核心缺口;建议核心回归优先使用本行(口径相对统一);【2026-08-25补充】泰山景区管委会官网(tsgw.taian.gov.cn)披露2022年1-8月进山游客179.51万人(非全年数据,不可直接填入缺口),与反推的2022全年基数214.8万大致吻合(该反推基期来自861.97这条数据,后已追溯确认为官方一手来源,见下方"已采纳"说明);【2026-08-25补充】官方确认2023年1-3月存在免门票政策,可能是当年游客量异常增长的部分原因,分析2023年数据时需注明此政策背景;【2026-08-25已采纳】2023年补充为861.97万人次,来源:泰山景区管委会官网《2023泰山景区答卷》(tsgw.taian.gov.cn,2024-01-03发布),官方一手来源,内部多个时间节点数据高度自洽,已存档archive/20260825_tsgw_2023_visitors_86197wan.md;唯一未解疑点:文中"比2019年增长106.41%"反推基数与统计局公报567.9万不符,可能因景区管委会内部口径与统计局口径存在细微差异,不影响对861.97本身的采信;【2026-08-25重大更新】2022年补充为214.8万人次,来源:上海新世纪资信评估投资服务有限公司《泰安市泰山投资有限公司跟踪评级报告》(2023-06-27),原文明确使用"进山进景点游客"表述,与本行2019/2021年统计口径一致(非另一套口径)。另,已找到关键澄清文件——《泰山景区安全隐患整治项目》专项债可行性报告(泰山景区管委会,2022年5月)原文写明"2018年...进山进景点游客、进山游客总人数562万人,其中进山总人数412万人":证实"进山进景点游客"(本行口径)与"进山总人数"(见下方新增行)是整体与子集关系,不是两套互相矛盾的口径,此前"口径切换"的判断需部分修正——本行2016-2023年实际上是同一套连续口径,只是逐年公报措辞不统一</t>
+          <t>【口径:进山/进泰山,不含非登顶访客】2019、2021年公报用词"进山进景点游客",2024、2025年用词"进泰山/进山游客量";2020年原文用词已核实(2026-08-26,PDF公报原文确认为"进山进景点游客278.6万",与主序列一致);2022、2023年公报未披露,仍为核心缺口;建议核心回归优先使用本行(口径相对统一);【2026-08-25补充】泰山景区管委会官网(tsgw.taian.gov.cn)披露2022年1-8月进山游客179.51万人(非全年数据,不可直接填入缺口),与反推的2022全年基数214.8万大致吻合(该反推基期来自861.97这条数据,后已追溯确认为官方一手来源,见下方"已采纳"说明);【2026-08-25补充】官方确认2023年1-3月存在免门票政策,可能是当年游客量异常增长的部分原因,分析2023年数据时需注明此政策背景;【2026-08-25已采纳】2023年补充为861.97万人次,来源:泰山景区管委会官网《2023泰山景区答卷》(tsgw.taian.gov.cn,2024-01-03发布),官方一手来源,内部多个时间节点数据高度自洽,已存档archive/20260825_tsgw_2023_visitors_86197wan.md;唯一未解疑点:文中"比2019年增长106.41%"反推基数与统计局公报567.9万不符,可能因景区管委会内部口径与统计局口径存在细微差异,不影响对861.97本身的采信;【2026-08-25重大更新】2022年补充为214.8万人次,来源:上海新世纪资信评估投资服务有限公司《泰安市泰山投资有限公司跟踪评级报告》(2023-06-27),原文明确使用"进山进景点游客"表述,与本行2019/2021年统计口径一致(非另一套口径)。另,已找到关键澄清文件——《泰山景区安全隐患整治项目》专项债可行性报告(泰山景区管委会,2022年5月)原文写明"2018年...进山进景点游客、进山游客总人数562万人,其中进山总人数412万人":证实"进山进景点游客"(本行口径)与"进山总人数"(见下方新增行)是整体与子集关系,不是两套互相矛盾的口径,此前"口径切换"的判断需部分修正——本行2016-2023年实际上是同一套连续口径,只是逐年公报措辞不统一
+【2026-09-17更正】2019/2020/2021/2024年颜色标记由"存疑"更正为"已核实"。依据：docs/data_priority_policy.md 案例三、八、九、十、十一、十二记录的多轮独立信源交叉核实（历年统计公报原文逐年措辞核对、专项债可行性报告、评级报告、景区管委会预算文件、以及用"较上年小幅减少"等定性描述做逻辑一致性排除法），该序列2016-2025年整条口径一致性与数值可信度已得到充分验证。此前颜色标记未同步更新，滞后于文字记录中已完成的核实工作，特此更正，不删除原有说明文字。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: correct unit label from 万人 to 万人次 for core visitor variable
泰山景区进山游客(窄口径)的单位由"万人"更正为"万人次"，涉及原始表、
数据字典、清洗数据表(xlsx+csv)、方法论笔记、两个核心脚本(py+ipynb)共9个文件；
冲突清单新增第10条记录此次更正
</commit_message>
<xml_diff>
--- a/data/raw/taian_indicators.xlsx
+++ b/data/raw/taian_indicators.xlsx
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>万人</t>
+          <t>万人次</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -1505,7 +1505,8 @@
       <c r="M8" s="8" t="inlineStr">
         <is>
           <t>【口径:进山/进泰山,不含非登顶访客】2019、2021年公报用词"进山进景点游客",2024、2025年用词"进泰山/进山游客量";2020年原文用词已核实(2026-08-26,PDF公报原文确认为"进山进景点游客278.6万",与主序列一致);2022、2023年公报未披露,仍为核心缺口;建议核心回归优先使用本行(口径相对统一);【2026-08-25补充】泰山景区管委会官网(tsgw.taian.gov.cn)披露2022年1-8月进山游客179.51万人(非全年数据,不可直接填入缺口),与反推的2022全年基数214.8万大致吻合(该反推基期来自861.97这条数据,后已追溯确认为官方一手来源,见下方"已采纳"说明);【2026-08-25补充】官方确认2023年1-3月存在免门票政策,可能是当年游客量异常增长的部分原因,分析2023年数据时需注明此政策背景;【2026-08-25已采纳】2023年补充为861.97万人次,来源:泰山景区管委会官网《2023泰山景区答卷》(tsgw.taian.gov.cn,2024-01-03发布),官方一手来源,内部多个时间节点数据高度自洽,已存档archive/20260825_tsgw_2023_visitors_86197wan.md;唯一未解疑点:文中"比2019年增长106.41%"反推基数与统计局公报567.9万不符,可能因景区管委会内部口径与统计局口径存在细微差异,不影响对861.97本身的采信;【2026-08-25重大更新】2022年补充为214.8万人次,来源:上海新世纪资信评估投资服务有限公司《泰安市泰山投资有限公司跟踪评级报告》(2023-06-27),原文明确使用"进山进景点游客"表述,与本行2019/2021年统计口径一致(非另一套口径)。另,已找到关键澄清文件——《泰山景区安全隐患整治项目》专项债可行性报告(泰山景区管委会,2022年5月)原文写明"2018年...进山进景点游客、进山游客总人数562万人,其中进山总人数412万人":证实"进山进景点游客"(本行口径)与"进山总人数"(见下方新增行)是整体与子集关系,不是两套互相矛盾的口径,此前"口径切换"的判断需部分修正——本行2016-2023年实际上是同一套连续口径,只是逐年公报措辞不统一
-【2026-09-17更正】2019/2020/2021/2024年颜色标记由"存疑"更正为"已核实"。依据：docs/data_priority_policy.md 案例三、八、九、十、十一、十二记录的多轮独立信源交叉核实（历年统计公报原文逐年措辞核对、专项债可行性报告、评级报告、景区管委会预算文件、以及用"较上年小幅减少"等定性描述做逻辑一致性排除法），该序列2016-2025年整条口径一致性与数值可信度已得到充分验证。此前颜色标记未同步更新，滞后于文字记录中已完成的核实工作，特此更正，不删除原有说明文字。</t>
+【2026-09-17更正】2019/2020/2021/2024年颜色标记由"存疑"更正为"已核实"。依据：docs/data_priority_policy.md 案例三、八、九、十、十一、十二记录的多轮独立信源交叉核实（历年统计公报原文逐年措辞核对、专项债可行性报告、评级报告、景区管委会预算文件、以及用"较上年小幅减少"等定性描述做逻辑一致性排除法），该序列2016-2025年整条口径一致性与数值可信度已得到充分验证。此前颜色标记未同步更新，滞后于文字记录中已完成的核实工作，特此更正，不删除原有说明文字。
+【2026-09-29更正】单位由"万人"更正为"万人次"。依据：本行说明中2022、2023年具体数字的引用均写作"万人次"（如"861.97万人次""214.8万人次"），与单位栏原标注的"万人"不一致；同一工作表内其他游客类指标（国内游客人次、接待游客总人次）单位均为"人次"。综合判断原单位栏"万人"为填写疏漏，更正为"万人次"。此前基于"万人"单位标注的下游文件（数据字典、清洗数据表、分析脚本等）已同步更正。</t>
         </is>
       </c>
     </row>

</xml_diff>